<commit_message>
Remediate SAP populations and bind full release pipeline
</commit_message>
<xml_diff>
--- a/03_metadata/adam/ADaM_spec.xlsx
+++ b/03_metadata/adam/ADaM_spec.xlsx
@@ -1349,12 +1349,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>SDTM.DM.ETHNIC.</t>
+          <t>Not collected in the public SDTM.DM release; assigned NOT REPORTED with the disposition documented in ADRG §5.1.</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Actual treatment assignment from first non-missing SDTM.EX exposure record and config/study_config.yaml treatment map.</t>
+          <t>Actual treatment assignment from SDTM.DM.ARM/ARMCD using the same Path A arm authority as TRT01P; EXTRT is not used because F-028 documents an inconsistent exposure treatment value.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Numeric actual treatment assignment from first non-missing SDTM.EX exposure record and config/study_config.yaml treatment map.</t>
+          <t>Numeric actual treatment assignment from SDTM.DM.ARM/ARMCD using the same Path A arm authority as TRT01PN; EXTRT is not used because F-028 documents an inconsistent exposure treatment value.</t>
         </is>
       </c>
     </row>
@@ -2453,7 +2453,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Baseline albumin from SDTM.LB records.</t>
+          <t>Not collected in the public SDTM.LB release; left missing with a blank imputation flag (ADRG §5.1).</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Baseline lactate dehydrogenase from SDTM.LB records.</t>
+          <t>Not collected in the public SDTM.LB release; left missing with a blank imputation flag (ADRG §5.1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align clinical simulation with FDA standards
</commit_message>
<xml_diff>
--- a/03_metadata/adam/ADaM_spec.xlsx
+++ b/03_metadata/adam/ADaM_spec.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study" sheetId="1" r:id="R8417359375c7412e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="R157960e7de3e429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="3" r:id="R7ba54f32b8544e54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValueLevel" sheetId="4" r:id="R342ecab52a594eef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhereClauses" sheetId="5" r:id="Rb6c7b016bfba4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelists" sheetId="6" r:id="R676e14af20e64810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionaries" sheetId="7" r:id="R339fe328673e42a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="8" r:id="R4f84911ab6864d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comments" sheetId="9" r:id="R260fc5554cf64d02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb45df35fb9364064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study" sheetId="1" r:id="Rc041649ab5554055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="Rcc20954077054d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="3" r:id="R2d217589ce264202"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValueLevel" sheetId="4" r:id="R717134b3794c4374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhereClauses" sheetId="5" r:id="R3109866325c14908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelists" sheetId="6" r:id="R93ff3ae7674a4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionaries" sheetId="7" r:id="Rb3c15e576fc749fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="8" r:id="R83a45a79b9d14a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comments" sheetId="9" r:id="Rb5b31fd95c3d44df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R449dfa3fdd8c48d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7368,15 +7368,11 @@
           <x:t xml:space="preserve">ADLB</x:t>
         </x:is>
       </x:c>
-      <x:c r="C124" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BASEFL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D124" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Baseline Record Flag</x:t>
-        </x:is>
+      <x:c r="C124" s="7" t="str">
+        <x:v>ABLFL</x:v>
+      </x:c>
+      <x:c r="D124" s="7" t="str">
+        <x:v>Baseline Record Flag</x:v>
       </x:c>
       <x:c r="E124" s="7" t="inlineStr">
         <x:is>
@@ -7404,13 +7400,11 @@
         </x:is>
       </x:c>
       <x:c r="L124" s="7" t="n"/>
-      <x:c r="M124" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MT.ADLB_BASEFL</x:t>
-        </x:is>
+      <x:c r="M124" s="7" t="str">
+        <x:v>MT.ADLB_ABLFL</x:v>
       </x:c>
       <x:c r="N124" s="7" t="str">
-        <x:v>Y only on the SDTM.LB record selected as baseline from LBBLFL=Y; N otherwise.</x:v>
+        <x:v>Y only on the deterministic SDTM.LB record selected as baseline from LBBLFL=Y; null otherwise.</x:v>
       </x:c>
       <x:c r="O124" s="7" t="n"/>
       <x:c r="P124" s="7" t="n"/>
@@ -13414,15 +13408,11 @@
       <x:c r="H35" s="7" t="n"/>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
-      <x:c r="A36" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MT.ADLB_BASEFL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B36" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Method for ADLB_BASEFL</x:t>
-        </x:is>
+      <x:c r="A36" s="7" t="str">
+        <x:v>MT.ADLB_ABLFL</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="str">
+        <x:v>Method for ADLB_ABLFL</x:v>
       </x:c>
       <x:c r="C36" s="7" t="inlineStr">
         <x:is>
@@ -13430,7 +13420,7 @@
         </x:is>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>Y only on the SDTM.LB record selected as baseline from LBBLFL=Y; N otherwise.</x:v>
+        <x:v>Y only on the deterministic SDTM.LB record selected as baseline from LBBLFL=Y; null otherwise.</x:v>
       </x:c>
       <x:c r="E36" s="7" t="n"/>
       <x:c r="F36" s="7" t="n"/>

</xml_diff>